<commit_message>
Fix 2025–2026 import price units for Petrobras crude imports
Use ANP ie.xlsx dispendio already denominated in USD when deriving
unit import prices for the YTD years.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/anp/petrobras_importacao_petroleo/petrobras_importacao_petroleo_2011_2026.xlsx
+++ b/anp/petrobras_importacao_petroleo/petrobras_importacao_petroleo_2011_2026.xlsx
@@ -865,17 +865,17 @@
         <v>47997500</v>
       </c>
       <c r="E16" t="n">
-        <v>73560439.47048666</v>
+        <v>73.56043947048666</v>
       </c>
       <c r="F16" t="n">
-        <v>3530717193484684</v>
+        <v>3530717193.484684</v>
       </c>
       <c r="G16" t="b">
         <v>0</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ANP ie.xlsx (dispêndio÷volume Brasil)</t>
+          <t>ANP ie.xlsx dispêndio÷volume</t>
         </is>
       </c>
     </row>
@@ -893,17 +893,17 @@
         <v>14326250</v>
       </c>
       <c r="E17" t="n">
-        <v>43824352.37465155</v>
+        <v>43.82435237465155</v>
       </c>
       <c r="F17" t="n">
-        <v>627838628207351.8</v>
+        <v>627838628.2073518</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ANP ie.xlsx (dispêndio÷volume Brasil)</t>
+          <t>ANP ie.xlsx dispêndio÷volume</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4158658878730295</v>
+        <v>107215594081.7221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>